<commit_message>
Split objective and behavioral-design intervention columns in status matrix
Rename "Objetivo" to "Objetivo del proyecto" and add "Intervención de diseño
de conducta" (the concrete behavioral lever/artifact designed per initiative).
Restyle for the new column layout and document both fields in the legend sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WS4JWEE6ms3s7RzgD4pkSb
</commit_message>
<xml_diff>
--- a/reportes/Status_Proyectos_Behavioral_Design.xlsx
+++ b/reportes/Status_Proyectos_Behavioral_Design.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Leyenda y notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$O$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -143,7 +143,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -513,23 +513,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="52" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -546,7 +547,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Clave</t>
@@ -564,55 +565,60 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Objetivo</t>
+          <t>Objetivo del proyecto</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>Intervención de diseño de conducta</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Estado (Jira)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Status (detalle)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>% Avance</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Equipo que requiere el servicio</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Stakeholder</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Equipo Behavioral Design</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Fichas</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Fecha de cierre</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Riesgos</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Impacto esperado</t>
         </is>
@@ -639,48 +645,53 @@
           <t>Promover el entendimiento y uso eficiente de los seguros de salud</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Guías resumidas/simplificadas de pólizas: rediseño de la información del producto para hacerla clara y comprensible (ataca la barrera de «falta de información»).</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>WIP - Documento de primer producto en agencia</t>
         </is>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="H5" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>AMI – Salud (Producto)</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Estrella Damian, Soiky Bardales</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Stef, Felipe, Alejandro</t>
         </is>
       </c>
-      <c r="K5" s="8" t="n">
+      <c r="L5" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>30 de junio</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Cambio en el roadmap (de 1 guía a 4 productos)</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>↓ ~25–30% casos NPS «no recibí información» (est.); ataca la palanca #1 de desconfianza en Perú</t>
         </is>
@@ -707,48 +718,53 @@
           <t>Reducir el churn y reclamos por cambios en la renovación</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Carta de renovación + batería de 3 soluciones de diseño en el momento de renovación; comunicación proactiva que reduce incertidumbre y fricción ante el cambio.</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Carta de renovación implementada; 3 soluciones diseñadas on hold</t>
         </is>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="H6" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>AMI – Renovación / Salud</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Estrella Damian, Soiky Bardales</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Alejandro</t>
         </is>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="L6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>30 de junio</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>La carta por sí sola no cubre la necesidad del usuario</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>+3–5 pp retención sobre base industria ~84% y ↓ reclamos (est.); depende de desbloquear las 3 soluciones on hold</t>
         </is>
@@ -775,48 +791,53 @@
           <t>Promover el entendimiento y uso eficiente de los seguros de salud</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Guías resumidas de pólizas para clientes corporativos TOP EPS; misma palanca de claridad/comprensión aplicada a cuentas clave.</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Implementado</t>
         </is>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="H7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>EPS – Salud Corporativa</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Kevin Crisanto, María Alejandra Valcarcel</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Stef, Felipe, Alejandro</t>
         </is>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="L7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>Producto pide no comunicar algunos servicios valorados por el usuario</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="O7" s="5" t="inlineStr">
         <is>
           <t>Renovación de cuentas TOP EPS (incl. Antapacay) + ↓ «no recibí información» en corporativo; alto valor por cuenta</t>
         </is>
@@ -843,48 +864,53 @@
           <t>Promover la captura de datos para conciliación de facturas proveedores</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Rediseño del flujo de captura de datos (Evolution+) para facilitar/incentivar que los proveedores entreguen la información de conciliación.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>En fase de research</t>
         </is>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="H8" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Cobranzas / Finanzas</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Rosemary Moyano</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Stef</t>
         </is>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="L8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>30 de junio</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>Track de diseño aprobado sin explorar la problemática</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="O8" s="5" t="inlineStr">
         <is>
           <t>Liberación de S/600k provisionados</t>
         </is>
@@ -911,48 +937,53 @@
           <t>Promover el agendamiento de citas comerciales</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Mensajes de primer contacto (copys/secuencia) que enmarcan la propuesta y reducen la fricción para agendar una cita comercial.</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>To Do (Block)</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Block</t>
         </is>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="H9" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Alejandro</t>
         </is>
       </c>
-      <c r="K9" s="8" t="n">
+      <c r="L9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>No existe estrategia definida de contacto bajo contexto CUA (bloqueado)</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>+20–30% agendamiento de citas en primer contacto (est., potencial — bloqueado por estrategia CUA)</t>
         </is>
@@ -979,48 +1010,53 @@
           <t>Diseñar un programa de lealtad del ecosistema que asegure la permanencia de los asegurados</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Diseño del programa de lealtad (mecánica de recompensas/beneficios) para reforzar la permanencia y el comportamiento de continuidad del asegurado.</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Diseñando y viabilizando la propuesta MVP/piloto (3–6 meses)</t>
         </is>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="H10" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Loyalty / Ecosistema RIMAC</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Denisse Galvez, Lucía Ramos, Jorge Sarmiento</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Alejandro</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="L10" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="O10" s="5" t="inlineStr">
         <is>
           <t>Permanencia base RIMAC (1,250 MM clientes); benchmark loyalty +20–25% retención y +40% cross-sell (est.)</t>
         </is>
@@ -1047,48 +1083,53 @@
           <t>Acelerar la curva de aprendizaje de asesores nuevos / mejorar ratio de conversión</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Programa de formación «Universidad Vida» para asesores nuevos: acelera la curva de aprendizaje con práctica estructurada.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>WIP</t>
         </is>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="H11" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Melissa, Alejandro</t>
         </is>
       </c>
-      <c r="K11" s="8" t="n">
+      <c r="L11" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>Capacidad limitada del equipo de learning</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr">
         <is>
           <t>−25–40% tiempo de ramp-up de asesores jr + mejor conversión y NPS Venta (est.)</t>
         </is>
@@ -1112,51 +1153,56 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Promover el aprendizaje y capacitación de asesores y dar visibilidad de expertise a jefaturas FFVV. Agente con el que el asesor practica casos; genera puntaje de efectividad y alertas por falta de principios básicos de experiencia (CX), visibles a jefaturas FFVV.</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
+          <t>Promover el aprendizaje y capacitación de asesores y dar visibilidad de expertise a jefaturas FFVV</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Agente entrenador (bot) de práctica de casos con puntaje de efectividad y alertas por falta de principios básicos de experiencia (CX); práctica deliberada con feedback y visibilidad a jefaturas.</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>In Review</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Prototipo diseñado y validada usabilidad y valoración de usuarios</t>
         </is>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="H12" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Felipe, Melissa</t>
         </is>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="L12" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>AIDA no cumple el task; entra a comité de priorización; 3 herramientas en paralelo</t>
         </is>
       </c>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>+efectividad del asesor (medible vía el puntaje del bot) y consistencia CX; práctica con feedback acelera ramp (−25–40%, est.); jefaturas hacen coaching dirigido. Ahorro proyectado S/1.8M (cifra del board, base por documentar)</t>
         </is>
@@ -1183,48 +1229,53 @@
           <t>Promover la generación de leads y agendamientos para FFVV</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Kit de social selling (contenido + herramientas de huella digital) para que la FFVV genere leads y agendamientos.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>WIP</t>
         </is>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="H13" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>Melissa</t>
         </is>
       </c>
-      <c r="K13" s="8" t="n">
+      <c r="L13" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>Recursos limitados de contenido + falta de incentivos + falta de monitoreo</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="O13" s="5" t="inlineStr">
         <is>
           <t>+leads/agendamientos FFVV; social selling 15–25% conversión lead→cita, CPL −30–50% (est.)</t>
         </is>
@@ -1251,62 +1302,67 @@
           <t>Piloto con colaboradores Rimac para construir hábitos saludables sostenibles</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Programa de hábitos saludables (piloto Bienestar 360) para construir y sostener hábitos de bienestar en colaboradores.</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="G14" s="7" t="n">
+      <c r="H14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Bienestar / Estar Bien</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Erika Echegaray, Belem Rodríguez; Solange Soto, Rosa Díaz</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>— (Equipo Bienestar / Estar Bien)</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Setiembre 2026 (solo acompañamiento)</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>Presupuesto y recursos limitados para la siguiente versión</t>
         </is>
       </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="O14" s="5" t="inlineStr">
         <is>
           <t>+3 ptos Wellby · CSAT 4.6/5 · NPS 78</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N14"/>
+  <autoFilter ref="A4:O14"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G14">
+  <conditionalFormatting sqref="H5:H14">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1325,11 +1381,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1339,7 +1395,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="44" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Fecha de corte</t>
@@ -1351,97 +1407,121 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="44" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
+          <t>Objetivo del proyecto</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>El para qué de negocio de la iniciativa (resultado buscado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Intervención de diseño de conducta</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>La solución/artefacto de behavioral design que se diseña e implementa: la palanca conductual concreta (guía, mensaje, programa, bot, kit, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
           <t>% Avance</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Estimación derivada del estado/status de cada iniciativa (no es un % reportado por el equipo). Done/Mantenimiento = 100%; In Review = 80%; In Progress = 20–40% según detalle; Block = 10%. Ajustar con el avance real de cada líder.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Equipo que requiere el servicio</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Campo inferido a partir del stakeholder y la iniciativa (área de negocio cliente del servicio de Behavioral Design). Confirmar con el equipo.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Stakeholder</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Tomado del board original (Behavioral_Design.pdf).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Equipo Behavioral Design</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Behavioral designers asignados (assignees).</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Fichas</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Capacidad asignada (8 de 10 fichas comprometibles por persona). Distribución propuesta, pendiente de confirmación. Alerta de capacidad: Alejandro 9/8 (🔴 sobreasignado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Capacidad asignada (8 de 10 fichas comprometibles por persona). Distribución propuesta, pendiente de confirmación. Alerta de capacidad: Alejandro 9/8 (sobreasignado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>(est.) en Impacto</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Estimación basada en benchmarks de industria + investigación interna del repo, no cifra comprometida por RIMAC.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Cifras duras</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Q-4 (S/600k), Q-8 (S/1.8M) y Q-10 (Wellby/CSAT/NPS) provienen del board original.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Estados (colores)</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Verde = Done · Azul = In Review · Amarillo = In Progress · Rojo = To Do (Block).</t>
         </is>

</xml_diff>

<commit_message>
Sync status matrix with team's working Excel
Add Prioridad column, rename Fecha de cierre -> Fecha de entrega, and add four
BD-capability initiatives (Q-11..Q-14, Chapter BD). Apply the team's field
updates (statuses, % avance, Q-10 now Stef/3 fichas, status detail, wording).
Fix obvious typos and complete Q-11's truncated impact; document all in the
legend sheet, including the capacity flag (Stef 11 fichas > 10).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WS4JWEE6ms3s7RzgD4pkSb
</commit_message>
<xml_diff>
--- a/reportes/Status_Proyectos_Behavioral_Design.xlsx
+++ b/reportes/Status_Proyectos_Behavioral_Design.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Leyenda y notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$O$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$P$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -52,7 +52,7 @@
       <color rgb="001F3864"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
       </patternFill>
     </fill>
     <fill>
@@ -111,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +145,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -513,24 +521,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
-    <col width="48" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -543,7 +552,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cierre Q2 2026 · Fecha de corte: 2026-06-22 · 6 épicas · 10 iniciativas</t>
+          <t>Cierre Q2 2026 · Fecha de corte: 2026-06-22 · 14 iniciativas (10 de negocio + 4 de capacidades del equipo BD)</t>
         </is>
       </c>
     </row>
@@ -565,60 +574,65 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>Objetivo del proyecto</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Intervención de diseño de conducta</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Estado (Jira)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Status (detalle)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>% Avance</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Equipo que requiere el servicio</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Stakeholder</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Equipo Behavioral Design</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Fichas</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Fecha de cierre</t>
-        </is>
-      </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
+          <t>Fecha de entrega</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
           <t>Riesgos</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Impacto esperado</t>
         </is>
@@ -642,56 +656,61 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
           <t>Promover el entendimiento y uso eficiente de los seguros de salud</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Guías resumidas/simplificadas de pólizas: rediseño de la información del producto para hacerla clara y comprensible (ataca la barrera de «falta de información»).</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Rediseño de la información del producto para hacerla clara y comprensible (ataca la barrera de «falta de información»).</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>WIP - Documento de primer producto en agencia</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>WIP - 1 producto en agencia</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>AMI – Salud (Producto)</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Estrella Damian, Soiky Bardales</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>Stef, Felipe, Alejandro</t>
         </is>
       </c>
-      <c r="L5" s="8" t="n">
+      <c r="M5" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>30 de junio</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Cambio en el roadmap (de 1 guía a 4 productos)</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>↓ ~25–30% casos NPS «no recibí información» (est.); ataca la palanca #1 de desconfianza en Perú</t>
         </is>
@@ -715,56 +734,61 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
           <t>Reducir el churn y reclamos por cambios en la renovación</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Carta de renovación + batería de 3 soluciones de diseño en el momento de renovación; comunicación proactiva que reduce incertidumbre y fricción ante el cambio.</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Comunicación proactiva que reduce incertidumbre y fricción ante el cambio.</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Diseñado</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Carta de renovación implementada; 3 soluciones diseñadas on hold</t>
         </is>
       </c>
-      <c r="H6" s="7" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>AMI – Renovación / Salud</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Estrella Damian, Soiky Bardales</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Alejandro</t>
         </is>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="M6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>30 de junio</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>La carta por sí sola no cubre la necesidad del usuario</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>+3–5 pp retención sobre base industria ~84% y ↓ reclamos (est.); depende de desbloquear las 3 soluciones on hold</t>
         </is>
@@ -788,56 +812,61 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
           <t>Promover el entendimiento y uso eficiente de los seguros de salud</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Guías resumidas de pólizas para clientes corporativos TOP EPS; misma palanca de claridad/comprensión aplicada a cuentas clave.</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Misma palanca de claridad/comprensión aplicada a cuentas clave.</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Implementado</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>1 implementada, 4 entregadas</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>EPS – Salud Corporativa</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Kevin Crisanto, María Alejandra Valcarcel</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
         <is>
           <t>Stef, Felipe, Alejandro</t>
         </is>
       </c>
-      <c r="L7" s="8" t="n">
+      <c r="M7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="O7" s="5" t="inlineStr">
         <is>
           <t>Producto pide no comunicar algunos servicios valorados por el usuario</t>
         </is>
       </c>
-      <c r="O7" s="5" t="inlineStr">
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>Renovación de cuentas TOP EPS (incl. Antapacay) + ↓ «no recibí información» en corporativo; alto valor por cuenta</t>
         </is>
@@ -861,56 +890,61 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
           <t>Promover la captura de datos para conciliación de facturas proveedores</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Rediseño del flujo de captura de datos (Evolution+) para facilitar/incentivar que los proveedores entreguen la información de conciliación.</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>En fase de research</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="I8" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Cobranzas / Finanzas</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Rosemary Moyano</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>Stef</t>
         </is>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="M8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>30 de junio</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="O8" s="5" t="inlineStr">
         <is>
           <t>Track de diseño aprobado sin explorar la problemática</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr">
+      <c r="P8" s="5" t="inlineStr">
         <is>
           <t>Liberación de S/600k provisionados</t>
         </is>
@@ -934,56 +968,61 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
           <t>Promover el agendamiento de citas comerciales</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Mensajes de primer contacto (copys/secuencia) que enmarcan la propuesta y reducen la fricción para agendar una cita comercial.</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>To Do (Block)</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Block</t>
         </is>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="I9" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>Alejandro</t>
         </is>
       </c>
-      <c r="L9" s="8" t="n">
+      <c r="M9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>No existe estrategia definida de contacto bajo contexto CUA (bloqueado)</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr">
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>+20–30% agendamiento de citas en primer contacto (est., potencial — bloqueado por estrategia CUA)</t>
         </is>
@@ -1007,56 +1046,61 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
           <t>Diseñar un programa de lealtad del ecosistema que asegure la permanencia de los asegurados</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Diseño del programa de lealtad (mecánica de recompensas/beneficios) para reforzar la permanencia y el comportamiento de continuidad del asegurado.</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Diseñando y viabilizando la propuesta MVP/piloto (3–6 meses)</t>
         </is>
       </c>
-      <c r="H10" s="7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Loyalty / Ecosistema RIMAC</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Denisse Galvez, Lucía Ramos, Jorge Sarmiento</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>Alejandro</t>
         </is>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="M10" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Julio 2026</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>Permanencia base RIMAC (1,250 MM clientes); benchmark loyalty +20–25% retención y +40% cross-sell (est.)</t>
         </is>
@@ -1080,56 +1124,61 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
           <t>Acelerar la curva de aprendizaje de asesores nuevos / mejorar ratio de conversión</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Programa de formación «Universidad Vida» para asesores nuevos: acelera la curva de aprendizaje con práctica estructurada.</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>WIP</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="n">
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Diseñado</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Contenido listo, falta diseño instruccional (Learning)</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>Melissa, Alejandro</t>
         </is>
       </c>
-      <c r="L11" s="8" t="n">
+      <c r="M11" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr">
         <is>
           <t>Capacidad limitada del equipo de learning</t>
         </is>
       </c>
-      <c r="O11" s="5" t="inlineStr">
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>−25–40% tiempo de ramp-up de asesores jr + mejor conversión y NPS Venta (est.)</t>
         </is>
@@ -1153,56 +1202,61 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
           <t>Promover el aprendizaje y capacitación de asesores y dar visibilidad de expertise a jefaturas FFVV</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Agente entrenador (bot) de práctica de casos con puntaje de efectividad y alertas por falta de principios básicos de experiencia (CX); práctica deliberada con feedback y visibilidad a jefaturas.</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>In Review</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Prototipo diseñado y validada usabilidad y valoración de usuarios</t>
         </is>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="I12" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
         <is>
           <t>Felipe, Melissa</t>
         </is>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="M12" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>AIDA no cumple el task; entra a comité de priorización; 3 herramientas en paralelo</t>
         </is>
       </c>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="P12" s="5" t="inlineStr">
         <is>
           <t>+efectividad del asesor (medible vía el puntaje del bot) y consistencia CX; práctica con feedback acelera ramp (−25–40%, est.); jefaturas hacen coaching dirigido. Ahorro proyectado S/1.8M (cifra del board, base por documentar)</t>
         </is>
@@ -1226,56 +1280,61 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
           <t>Promover la generación de leads y agendamientos para FFVV</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Kit de social selling (contenido + herramientas de huella digital) para que la FFVV genere leads y agendamientos.</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>WIP</t>
         </is>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="I13" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>FFVV Vida Individual</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>Diana Riofrío, Jaime Huerta</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="L13" s="5" t="inlineStr">
         <is>
           <t>Melissa</t>
         </is>
       </c>
-      <c r="L13" s="8" t="n">
+      <c r="M13" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Julio 2026</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="O13" s="5" t="inlineStr">
         <is>
           <t>Recursos limitados de contenido + falta de incentivos + falta de monitoreo</t>
         </is>
       </c>
-      <c r="O13" s="5" t="inlineStr">
+      <c r="P13" s="5" t="inlineStr">
         <is>
           <t>+leads/agendamientos FFVV; social selling 15–25% conversión lead→cita, CPL −30–50% (est.)</t>
         </is>
@@ -1299,70 +1358,393 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
           <t>Piloto con colaboradores Rimac para construir hábitos saludables sostenibles</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Programa de hábitos saludables (piloto Bienestar 360) para construir y sostener hábitos de bienestar en colaboradores.</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Mantenimiento</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Implementado y en mantenimiento</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Bienestar / Estar Bien</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>Erika Echegaray, Belem Rodríguez; Solange Soto, Rosa Díaz</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>— (Equipo Bienestar / Estar Bien)</t>
-        </is>
-      </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Stef</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Setiembre 2026 (solo acompañamiento)</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Presupuesto y recursos limitados para la siguiente versión</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>+3 ptos Wellby · CSAT 4.6/5 · NPS 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Q-11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Modelo de entendimiento y uso eficiente de seguros</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura BD</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Capacidades equipo BD</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Definir framework de trabajo para ecosistema de entendimiento y uso eficiente de seguros</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura del conocimiento</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Terminado el framework de trabajo; falta alinear con los distintos frentes involucrados</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Chapter BD</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>Setiembre 2026 (solo acompañamiento)</t>
-        </is>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>Presupuesto y recursos limitados para la siguiente versión</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>+3 ptos Wellby · CSAT 4.6/5 · NPS 78</t>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Framework para potenciar el entendimiento y uso eficiente de seguros</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Q-12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Sistema de generación de usuarios sintéticos</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura BD</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Capacidades equipo BD</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Crear recurso de exploración para conocimiento esencial de seguros y comportamiento con los seguros en Perú</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Creación de herramienta de testeo</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Diseñado</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Terminado, por validar</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Chapter BD</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Agilidad en el testeo de preguntas ya exploradas sobre conducta con seguros</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Q-13</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Modelo de cambio de hábitos</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura BD</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Capacidades equipo BD</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Definir framework de trabajo para ecosistema de entendimiento y uso eficiente de seguros</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura del conocimiento</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Terminado y validado</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Chapter BD</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Framework para trabajo de iniciativas relacionadas al cambio de hábitos</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Q-14</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Skill para desk research con rigurosidad científica</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Arquitectura BD</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Capacidades equipo BD</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Potenciar el desk research con parámetros de búsqueda con rigurosidad metodológica y creación de repositorio de conocimiento</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Creación de herramienta de research</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Diseñado</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Terminado, por validar</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Chapter BD</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Agilidad y calidad de los entregables de investigación de escritorio</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O14"/>
+  <autoFilter ref="A4:P18"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H14">
+  <conditionalFormatting sqref="I5:I18">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1381,11 +1763,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="92" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="94" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1395,135 +1777,159 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Fecha de corte</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-22. Sincronizado con el Excel de trabajo del equipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>«Priorizada por negocio» = demanda de un área cliente · «Capacidades equipo BD» = proyectos internos de arquitectura/herramientas del Chapter BD (Q-11 a Q-14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Objetivo del proyecto</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>El para qué de negocio de la iniciativa (resultado buscado).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Intervención de diseño de conducta</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>La solución/artefacto de behavioral design que se diseña e implementa: la palanca conductual concreta (guía, mensaje, programa, bot, kit, etc.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>La solución/artefacto de behavioral design que se diseña e implementa: la palanca conductual concreta (guía, mensaje, programa, bot, kit, framework, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>% Avance</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Estimación derivada del estado/status de cada iniciativa (no es un % reportado por el equipo). Done/Mantenimiento = 100%; In Review = 80%; In Progress = 20–40% según detalle; Block = 10%. Ajustar con el avance real de cada líder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="44" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Avance por iniciativa según el equipo (Excel de trabajo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Equipo que requiere el servicio</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Campo inferido a partir del stakeholder y la iniciativa (área de negocio cliente del servicio de Behavioral Design). Confirmar con el equipo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Área cliente del servicio de Behavioral Design. «Chapter BD» = trabajo interno del equipo (capacidades).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Stakeholder</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Tomado del board original (Behavioral_Design.pdf).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Tomado del board original. Las iniciativas de capacidades BD no tienen stakeholder externo (—).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Equipo Behavioral Design</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Behavioral designers asignados (assignees).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="44" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Behavioral designers asignados. «Todos» en las iniciativas de capacidades BD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Fichas</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Capacidad asignada (8 de 10 fichas comprometibles por persona). Distribución propuesta, pendiente de confirmación. Alerta de capacidad: Alejandro 9/8 (sobreasignado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Capacidad por iniciativa (regla 8/2). CAPACIDAD: con Q-10 asignado a Stef, Stef acumula 11 fichas (Q-1, Q-3, Q-4, Q-10) → supera el máximo de 10; Alejandro queda en 9 (sobreasignado). Revisar reasignación. Q-11 a Q-14 las trabaja «Todos» sin fichas asignadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>(est.) en Impacto</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Estimación basada en benchmarks de industria + investigación interna del repo, no cifra comprometida por RIMAC.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Cifras duras</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Q-4 (S/600k), Q-8 (S/1.8M) y Q-10 (Wellby/CSAT/NPS) provienen del board original.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="44" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Correcciones aplicadas</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Typos del Excel de trabajo: «escencial»→«esencial», «Aglidad»→«Agilidad», «cmabio»→«cambio», «cinetífica»→«científica». Impacto de Q-11 estaba truncado («…uso efic») y se completó a «…uso eficiente de seguros».</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Estados (colores)</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Verde = Done · Azul = In Review · Amarillo = In Progress · Rojo = To Do (Block).</t>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Verde = Done · Azul = In Review · Lila = Diseñado · Amarillo = In Progress · Rojo = To Do (Block).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update projects with Q3-2026 roadmap (Chapter SD1)
Sync both artifacts (Excel matrix + Beholder board) with the Q3-2026 roadmap:
update the 14 existing initiatives (status, dates, owners, sub-tasks) and add
12 new ones (Q-15..Q-26): Nuevo seguro AMI, MBI-Vivo, Evolution+ Reservas Vida
and AMI continuidad, Comunicaciones Loyalty, Modelo de relacionamiento
empresas, RIMAC Wrap, recordatorio multicanal, sistema de incentivos, nuevo
modelo de ventas, postventa, derivación MER. Flag garbled-PDF uncertainties
as "(por confirmar)", note conflicts (Q-3, Q-5) and the fichas capacity issue
(Stef 11 > 10).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WS4JWEE6ms3s7RzgD4pkSb
</commit_message>
<xml_diff>
--- a/reportes/Status_Proyectos_Behavioral_Design.xlsx
+++ b/reportes/Status_Proyectos_Behavioral_Design.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Leyenda y notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$P$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$P$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -71,6 +71,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E4DFEC"/>
       </patternFill>
     </fill>
@@ -81,12 +86,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -521,25 +521,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="46" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -552,7 +552,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cierre Q2 2026 · Fecha de corte: 2026-06-22 · 14 iniciativas (10 de negocio + 4 de capacidades del equipo BD)</t>
+          <t>Roadmap Q3-2026 (Chapter SD1) · Fecha de corte: 2026-06-22 · 26 iniciativas (14 previas + 12 nuevas del roadmap)</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>WIP - 1 producto en agencia</t>
+          <t>Diseño 1/4; roadmap reajustado −6 semanas; presentación del entregable 30/6; + flyers de venta (1×producto + comparativo)</t>
         </is>
       </c>
       <c r="I5" s="7" t="n">
@@ -702,12 +702,12 @@
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>30 de junio</t>
+          <t>30/06 (presentación)</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>Cambio en el roadmap (de 1 guía a 4 productos)</t>
+          <t>Cambio en el roadmap (de 1 guía a 4 productos); reajuste −6 semanas</t>
         </is>
       </c>
       <c r="P5" s="5" t="inlineStr">
@@ -744,21 +744,21 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Comunicación proactiva que reduce incertidumbre y fricción ante el cambio.</t>
+          <t>Comunicación proactiva que reduce incertidumbre y fricción ante el cambio (speeches de primer contacto + carta de renovación).</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Diseñado</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Carta de renovación implementada; 3 soluciones diseñadas on hold</t>
+          <t>Guía de comunicación con escenarios y speeches: entregada; feedback y ajustes finales. Carta de renovación: Oncológicos BBVA (diseño acotado implementado)</t>
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Guías resumidas — 5 clientes TOP EPS</t>
+          <t>Guías resumidas — EPS (Top 4 cuentas + Multiempresa)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -825,18 +825,18 @@
           <t>Misma palanca de claridad/comprensión aplicada a cuentas clave.</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>In Review</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>1 implementada, 4 entregadas</t>
+          <t>Top 4 cuentas: 2/4 entregadas, 2/4 en revisión; Multiempresa: entregada; ajustes del entregable y presentación final</t>
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
@@ -885,7 +885,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Captura de datos para conciliación de facturas de proveedores</t>
+          <t>Optimización de Cobranzas B2B</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>En fase de research</t>
+          <t>12 entrevistas brokers/clientes B2B (entendimiento E2E del pago, pains de confirmación) → bajada/análisis → diseño de la nueva experiencia y pilotos → ejecutar piloto y definir experiencia final</t>
         </is>
       </c>
       <c r="I8" s="7" t="n">
@@ -936,7 +936,7 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>30 de junio</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
@@ -981,18 +981,18 @@
           <t>Mensajes de primer contacto (copys/secuencia) que enmarcan la propuesta y reducen la fricción para agendar una cita comercial.</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>To Do (Block)</t>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Block</t>
+          <t>Estrategia de primer contacto alineado a CUA (en definición → desbloqueándose); speeches de primer contacto</t>
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>No existe estrategia definida de contacto bajo contexto CUA (bloqueado)</t>
+          <t>Estrategia de contacto bajo contexto CUA en definición (antes bloqueado)</t>
         </is>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>+20–30% agendamiento de citas en primer contacto (est., potencial — bloqueado por estrategia CUA)</t>
+          <t>+20–30% agendamiento de citas en primer contacto (est.)</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Programa de lealtad (MVP/piloto)</t>
+          <t>Programa de lealtad — Piloto/MVP</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Diseñando y viabilizando la propuesta MVP/piloto (3–6 meses)</t>
+          <t>Piloto/MVP: definición de operativa, niveles de beneficios y clientes participantes (Meli) → envío de solicitud + push de participantes (Meli) → inicio y soporte del piloto (Alejandro)</t>
         </is>
       </c>
       <c r="I10" s="7" t="n">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Alejandro</t>
+          <t>Meli, Alejandro</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>Julio 2026</t>
+          <t>Q3 2026 (piloto 24/08–08/09)</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1137,14 +1137,14 @@
           <t>Programa de formación «Universidad Vida» para asesores nuevos: acelera la curva de aprendizaje con práctica estructurada.</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="10" t="inlineStr">
         <is>
           <t>Diseñado</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Contenido listo, falta diseño instruccional (Learning)</t>
+          <t>Asistencia a onboarding de FFVV actual; contenido listo, falta diseño instruccional (Learning)</t>
         </is>
       </c>
       <c r="I11" s="7" t="n">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Skill AIDA Bot Trainer + reportería</t>
+          <t>Copiloto del Asesor: AIDA — Bot trainer + reportería</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1215,14 +1215,14 @@
           <t>Agente entrenador (bot) de práctica de casos con puntaje de efectividad y alertas por falta de principios básicos de experiencia (CX); práctica deliberada con feedback y visibilidad a jefaturas.</t>
         </is>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>In Review</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Prototipo diseñado y validada usabilidad y valoración de usuarios</t>
+          <t>Prototipo diseñado y validada usabilidad y valoración de usuarios; en track de Back to Basics | Venta Vida</t>
         </is>
       </c>
       <c r="I12" s="7" t="n">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Kit de social selling (contenido + herramientas de huella digital) para que la FFVV genere leads y agendamientos.</t>
+          <t>Estrategia y contenido del Social Selling (contenido + herramientas de huella digital) para que la FFVV genere leads y agendamientos.</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>WIP</t>
+          <t>Estrategia y contenido del Social Selling; en track de Back to Basics | Venta Vida</t>
         </is>
       </c>
       <c r="I13" s="7" t="n">
@@ -1371,14 +1371,14 @@
           <t>Programa de hábitos saludables (piloto Bienestar 360) para construir y sostener hábitos de bienestar en colaboradores.</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Implementado y en mantenimiento</t>
+          <t>Implementado y en mantenimiento; cierre de playbook del programa + acompañamiento a la fase de mantenimiento</t>
         </is>
       </c>
       <c r="I14" s="7" t="n">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Terminado el framework de trabajo; falta alinear con los distintos frentes involucrados</t>
+          <t>Framework de trabajo terminado; falta alinear con los distintos frentes involucrados. En roadmap Q3: Backlog (Arquitectura BD)</t>
         </is>
       </c>
       <c r="I15" s="7" t="n">
@@ -1529,14 +1529,14 @@
           <t>Creación de herramienta de testeo</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>Diseñado</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Terminado, por validar</t>
+          <t>Terminado, por validar. En roadmap Q3: Backlog (Arquitectura BD)</t>
         </is>
       </c>
       <c r="I16" s="7" t="n">
@@ -1609,14 +1609,14 @@
           <t>Arquitectura del conocimiento</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Terminado y validado</t>
+          <t>Terminado y validado. En roadmap Q3: Backlog (Arquitectura BD)</t>
         </is>
       </c>
       <c r="I17" s="7" t="n">
@@ -1689,14 +1689,14 @@
           <t>Creación de herramienta de research</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Diseñado</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Terminado, por validar</t>
+          <t>Terminado, por validar. En roadmap Q3: Backlog (Arquitectura BD)</t>
         </is>
       </c>
       <c r="I18" s="7" t="n">
@@ -1738,13 +1738,973 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Q-15</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo seguro AMI</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Nuevos planes AMI + Seguro PT/P</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Lanzar nuevos planes AMI con materiales de venta y capacitación a la FFVV</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Entrega de guías resumidas, carta de bienvenida, speech de venta y flyers; capacitación FFVV; lineamientos de experiencia de venta y siniestros (Seguro PT/P).</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Entrega 1ª guía (plan vital, maquetado de agencia), carta de bienvenida, speech de venta (Speech Analytics), flyer; apoyo en nombres de planes (Marketing); capacitación FFVV; seguimiento a lanzamiento. Seguro PT/P: lineamientos de experiencia (por confirmar)</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>AMI – Salud (Producto)</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Q-16</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Salud integral</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>MBI – Vivo (piloto)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Pilotear MBI – Vivo con un segmento definido con Salud / Estar Bien</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Diseño y aterrizaje de un piloto (propuesta, presupuesto, producción y lanzamiento).</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Presentación y revisión de la propuesta del piloto; retomar conversaciones con stakeholders (Salud / Estar Bien) para definir el segmento; definición de presupuesto; aterrizaje y aprobación; producción y lanzamiento del piloto</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Salud / Estar Bien</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Q-17</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Evolution+: Reservas Vida</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Negociación y liberación de reservas vida</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Liberar reservas de vida mediante una nueva experiencia de gestión</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Diseño de la experiencia vista cliente E2E (4 fases) + piloto + co-diseño del escalamiento.</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Diseño de la experiencia E2E en 4 fases; implementación del piloto; co-diseñar el escalamiento con el equipo de proceso; adecuar a gestión externa (Rimac empresa tercera); seguimiento al despliegue</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas / Vida</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Q-18</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Evolution+: AMI continuidad</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Optimización de venta nueva AMI con continuidad</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Optimizar la venta nueva AMI con continuidad</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Piloto de venta por el hub + actualización de viabilidad financiera + definición de escalamiento.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Implementación del piloto para venta por el hub; actualización de la viabilidad financiera (caída en venta vs costo potencial de atención); definición de escalamiento a otros frentes (brokers, online y VIP)</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>AMI – Salud / Comercial</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Q-19</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Comunicaciones Loyalty</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Diseño de piezas y journeys de comunicación</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Soportar Loyalty/Renovación con piezas y journeys de comunicación</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Diseño de piezas y journeys (Angio Hogar/Vida, Protección Múltiple, Venta Hospitalaria, Renovación, Cobranza transversal).</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Diseño de piezas y journeys: Angio Hogar Total, Seguro Reciclar (journey), Protección Múltiple / Venta Hospitalaria, Renovación / WhatsApp, Cobranza transversal (imagen Royal)</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Loyalty / Comunicaciones</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Q-20</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Loyalty Empresas</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Modelo de relacionamiento empresas + Propuesta de valor</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Priorizada por negocio</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Definir el modelo de relacionamiento y la propuesta de valor para empresas</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Talleres de ideación + benchmark + modelos de relacionamiento (directo, brokers, corporativo) + propuesta de valor.</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Taller de ideación (30/06 presencial Lima · 02/07 virtual provincia); modelos de relacionamiento empresas directo / brokers / corporativo (benchmark, análisis, entregable y presentación final); potenciar storytelling de la propuesta de valor (con Marketing)</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Loyalty / Empresas</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M24" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Q-21</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Renovación</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>RIMAC Wrap (tangibilización pre-renovación)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Backlog (Chapter SD1)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Tangibilizar el valor antes de la renovación</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Toque de tangibilización pre-renovación (RIMAC Wrap).</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Renovación</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Q-22</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Renovación</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Recordatorio multicanal (SMS/WhatsApp/Push)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Backlog (Chapter SD1)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Reforzar la renovación con recordatorios multicanal</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Toques adicionales de recordatorio multicanal (SMS, WhatsApp y Push Notifications).</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Renovación</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M26" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Q-23</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Venta</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Sistema de incentivos orientados a la experiencia</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Backlog (Chapter SD1)</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Orientar los incentivos de asesores hacia la experiencia</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Diseño de un sistema de incentivos para asesores orientado a la experiencia (Back to Basics).</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Venta</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Q-24</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo Modelo de Ventas</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Convenios y Financieros — nuevo modelo de venta</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Backlog (Chapter SD1)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Definir un nuevo modelo de venta para Convenios y Financieros</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo modelo de venta para Convenios y Financieros.</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Backlog del Chapter SD1. Convenios (sponsor Diana Riofrío y Patricia Romero); Financieros (sponsor Claro Gomez y Patricia Romero)</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Venta / Convenios y Financieros</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>Diana Riofrío, Patricia Romero (Convenios); Claro Gomez, Patricia Romero (Financieros)</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M28" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Q-25</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Vida Individual</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Experiencia Postventa</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Backlog (Chapter SD1)</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Mejorar la experiencia postventa de Vida Individual</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Rediseño de la experiencia postventa.</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Backlog del Chapter SD1 (sponsor Diana Riofrío)</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Vida Individual / Posventa</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>Diana Riofrío</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M29" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Q-26</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Ahorro Salud</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Derivación eficiente MER</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Backlog (Chapter SD1)</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Hacer más eficiente la derivación (MER) en Ahorro Salud</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Rediseño de la derivación eficiente MER.</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Ahorro Salud</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>(por confirmar)</t>
+        </is>
+      </c>
+      <c r="M30" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:P18"/>
+  <autoFilter ref="A4:P30"/>
   <mergeCells count="2">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I18">
+  <conditionalFormatting sqref="I5:I30">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1763,11 +2723,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="94" customWidth="1" min="2" max="2"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1777,159 +2737,171 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="46" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Fecha de corte</t>
+          <t>Fuente / corte</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>2026-06-22. Sincronizado con el Excel de trabajo del equipo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="46" customHeight="1">
+          <t>2026-06-22. Actualizado con el Roadmap Q3-2026 (Chapter SD1). El PDF del roadmap tenía el texto distorsionado; los campos inciertos van marcados «(por confirmar)».</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
+          <t>Conflictos detectados</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Q-3: el Excel previo decía «5 clientes / Done»; el roadmap dice «Top 4 cuentas (2/4 entregadas, 2/4 en revisión) + Multiempresa entregada» → quedó In Review. Q-5: estaba «To Do (Block)»; el roadmap muestra «Estrategia de primer contacto alineado a CUA» activa → pasó a In Progress (desbloqueándose). Confirmar ambos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Iniciativas nuevas (Q-15–Q-26)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Del roadmap Q3 Chapter SD1: Nuevo seguro AMI, MBI-Vivo, Evolution+ Reservas Vida, Evolution+ AMI continuidad, Comunicaciones Loyalty, Modelo de relacionamiento empresas, RIMAC Wrap, Recordatorio multicanal, Sistema de incentivos, Nuevo modelo de ventas Convenios/Financieros, Vida Individual Postventa, Derivación eficiente MER. Owners y fichas por asignar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
           <t>Prioridad</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>«Priorizada por negocio» = demanda de un área cliente · «Capacidades equipo BD» = proyectos internos de arquitectura/herramientas del Chapter BD (Q-11 a Q-14).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>«Priorizada por negocio» · «Capacidades equipo BD» (Q-11–Q-14) · «Backlog (Chapter SD1)» para iniciativas nuevas sin sprint asignado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Objetivo del proyecto</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>El para qué de negocio de la iniciativa (resultado buscado).</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Intervención de diseño de conducta</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>La solución/artefacto de behavioral design que se diseña e implementa: la palanca conductual concreta (guía, mensaje, programa, bot, kit, framework, etc.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>La solución/artefacto de behavioral design que se diseña: la palanca conductual concreta (guía, mensaje, programa, bot, kit, framework, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>% Avance</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Avance por iniciativa según el equipo (Excel de trabajo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Avance por iniciativa según el equipo / roadmap. Iniciativas nuevas: estimación inicial (por confirmar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Equipo que requiere el servicio</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Área cliente del servicio de Behavioral Design. «Chapter BD» = trabajo interno del equipo (capacidades).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Área cliente del servicio de BD. «Chapter BD» = trabajo interno (capacidades).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Stakeholder</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Tomado del board original. Las iniciativas de capacidades BD no tienen stakeholder externo (—).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Del board original / roadmap. Las nuevas iniciativas tienen stakeholder «(por confirmar)» salvo Convenios/Financieros (Diana Riofrío, Patricia Romero, Claro Gomez) y Postventa (Diana Riofrío).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Equipo Behavioral Design</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Behavioral designers asignados. «Todos» en las iniciativas de capacidades BD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Behavioral designers asignados. Loyalty (Q-6): Meli + Alejandro (según roadmap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Fichas</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Capacidad por iniciativa (regla 8/2). CAPACIDAD: con Q-10 asignado a Stef, Stef acumula 11 fichas (Q-1, Q-3, Q-4, Q-10) → supera el máximo de 10; Alejandro queda en 9 (sobreasignado). Revisar reasignación. Q-11 a Q-14 las trabaja «Todos» sin fichas asignadas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Capacidad por iniciativa (regla 8/2). PENDIENTE: Stef acumula 11 fichas (Q-1,Q-3,Q-4,Q-10) → supera el máximo de 10; Alejandro en 9 (sobreasignado). Las iniciativas nuevas (Q-15–Q-26) están sin fichas asignadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>(est.) en Impacto</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Estimación basada en benchmarks de industria + investigación interna del repo, no cifra comprometida por RIMAC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="46" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Estimación basada en benchmarks + investigación interna; no cifra comprometida por RIMAC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Cifras duras</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Q-4 (S/600k), Q-8 (S/1.8M) y Q-10 (Wellby/CSAT/NPS) provienen del board original.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Correcciones aplicadas</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Typos del Excel de trabajo: «escencial»→«esencial», «Aglidad»→«Agilidad», «cmabio»→«cambio», «cinetífica»→«científica». Impacto de Q-11 estaba truncado («…uso efic») y se completó a «…uso eficiente de seguros».</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="46" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Estados (colores)</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>Verde = Done · Azul = In Review · Lila = Diseñado · Amarillo = In Progress · Rojo = To Do (Block).</t>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Verde = Done · Azul = In Review · Lila = Diseñado · Amarillo = In Progress · Rojo = To Do (Block) · Gris = Backlog.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align Excel + board after Stefanie removed Q-17/Q-18
Regenerate the Excel matrix without Q-17/Q-18 (24 rows), fix the board's
count label (14 previas + 10 nuevas) and EPIC-4 title (now only Q-4), and
log the change in the 15-day history.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WS4JWEE6ms3s7RzgD4pkSb
</commit_message>
<xml_diff>
--- a/reportes/Status_Proyectos_Behavioral_Design.xlsx
+++ b/reportes/Status_Proyectos_Behavioral_Design.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Leyenda y notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$P$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Proyectos'!$A$4:$P$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Roadmap Q3-2026 (Chapter SD1) · Fecha de corte: 2026-06-22 · 26 iniciativas (14 previas + 12 nuevas del roadmap)</t>
+          <t>Roadmap Q3-2026 (Chapter SD1) · Fecha de corte: 2026-06-23 · 24 iniciativas (14 previas + 10 nuevas del roadmap)</t>
         </is>
       </c>
     </row>
@@ -1901,17 +1901,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Q-17</t>
+          <t>Q-19</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Evolution+: Reservas Vida</t>
+          <t>Comunicaciones Loyalty</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Negociación y liberación de reservas vida</t>
+          <t>Diseño de piezas y journeys de comunicación</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1921,12 +1921,12 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Liberar reservas de vida mediante una nueva experiencia de gestión</t>
+          <t>Soportar Loyalty/Renovación con piezas y journeys de comunicación</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Diseño de la experiencia vista cliente E2E (4 fases) + piloto + co-diseño del escalamiento.</t>
+          <t>Diseño de piezas y journeys (Angio Hogar/Vida, Protección Múltiple, Venta Hospitalaria, Renovación, Cobranza transversal).</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1936,15 +1936,15 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Diseño de la experiencia E2E en 4 fases; implementación del piloto; co-diseñar el escalamiento con el equipo de proceso; adecuar a gestión externa (Rimac empresa tercera); seguimiento al despliegue</t>
+          <t>Diseño de piezas y journeys: Angio Hogar Total, Seguro Reciclar (journey), Protección Múltiple / Venta Hospitalaria, Renovación / WhatsApp, Cobranza transversal (imagen Royal)</t>
         </is>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Finanzas / Vida</t>
+          <t>Loyalty / Comunicaciones</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -1981,17 +1981,17 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Q-18</t>
+          <t>Q-20</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Evolution+: AMI continuidad</t>
+          <t>Loyalty Empresas</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Optimización de venta nueva AMI con continuidad</t>
+          <t>Modelo de relacionamiento empresas + Propuesta de valor</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Optimizar la venta nueva AMI con continuidad</t>
+          <t>Definir el modelo de relacionamiento y la propuesta de valor para empresas</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Piloto de venta por el hub + actualización de viabilidad financiera + definición de escalamiento.</t>
+          <t>Talleres de ideación + benchmark + modelos de relacionamiento (directo, brokers, corporativo) + propuesta de valor.</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -2016,15 +2016,15 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Implementación del piloto para venta por el hub; actualización de la viabilidad financiera (caída en venta vs costo potencial de atención); definición de escalamiento a otros frentes (brokers, online y VIP)</t>
+          <t>Taller de ideación (30/06 presencial Lima · 02/07 virtual provincia); modelos de relacionamiento empresas directo / brokers / corporativo (benchmark, análisis, entregable y presentación final); potenciar storytelling de la propuesta de valor (con Marketing)</t>
         </is>
       </c>
       <c r="I22" s="7" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>AMI – Salud / Comercial</t>
+          <t>Loyalty / Empresas</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2061,50 +2061,50 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Q-19</t>
+          <t>Q-21</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Comunicaciones Loyalty</t>
+          <t>Renovación</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Diseño de piezas y journeys de comunicación</t>
+          <t>RIMAC Wrap (tangibilización pre-renovación)</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Priorizada por negocio</t>
+          <t>Backlog (Chapter SD1)</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Soportar Loyalty/Renovación con piezas y journeys de comunicación</t>
+          <t>Tangibilizar el valor antes de la renovación</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Diseño de piezas y journeys (Angio Hogar/Vida, Protección Múltiple, Venta Hospitalaria, Renovación, Cobranza transversal).</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+          <t>Toque de tangibilización pre-renovación (RIMAC Wrap).</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Diseño de piezas y journeys: Angio Hogar Total, Seguro Reciclar (journey), Protección Múltiple / Venta Hospitalaria, Renovación / WhatsApp, Cobranza transversal (imagen Royal)</t>
+          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
         </is>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Loyalty / Comunicaciones</t>
+          <t>Renovación</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
@@ -2141,50 +2141,50 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Q-20</t>
+          <t>Q-22</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Loyalty Empresas</t>
+          <t>Renovación</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Modelo de relacionamiento empresas + Propuesta de valor</t>
+          <t>Recordatorio multicanal (SMS/WhatsApp/Push)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Priorizada por negocio</t>
+          <t>Backlog (Chapter SD1)</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Definir el modelo de relacionamiento y la propuesta de valor para empresas</t>
+          <t>Reforzar la renovación con recordatorios multicanal</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Talleres de ideación + benchmark + modelos de relacionamiento (directo, brokers, corporativo) + propuesta de valor.</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+          <t>Toques adicionales de recordatorio multicanal (SMS, WhatsApp y Push Notifications).</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Taller de ideación (30/06 presencial Lima · 02/07 virtual provincia); modelos de relacionamiento empresas directo / brokers / corporativo (benchmark, análisis, entregable y presentación final); potenciar storytelling de la propuesta de valor (con Marketing)</t>
+          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
         </is>
       </c>
       <c r="I24" s="7" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Loyalty / Empresas</t>
+          <t>Renovación</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>Q3 2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -2221,17 +2221,17 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Q-21</t>
+          <t>Q-23</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Renovación</t>
+          <t>Venta</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>RIMAC Wrap (tangibilización pre-renovación)</t>
+          <t>Sistema de incentivos orientados a la experiencia</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -2241,12 +2241,12 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Tangibilizar el valor antes de la renovación</t>
+          <t>Orientar los incentivos de asesores hacia la experiencia</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Toque de tangibilización pre-renovación (RIMAC Wrap).</t>
+          <t>Diseño de un sistema de incentivos para asesores orientado a la experiencia (Back to Basics).</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Renovación</t>
+          <t>Venta</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
@@ -2301,17 +2301,17 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Q-22</t>
+          <t>Q-24</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Renovación</t>
+          <t>Nuevo Modelo de Ventas</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Recordatorio multicanal (SMS/WhatsApp/Push)</t>
+          <t>Convenios y Financieros — nuevo modelo de venta</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -2321,12 +2321,12 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Reforzar la renovación con recordatorios multicanal</t>
+          <t>Definir un nuevo modelo de venta para Convenios y Financieros</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Toques adicionales de recordatorio multicanal (SMS, WhatsApp y Push Notifications).</t>
+          <t>Nuevo modelo de venta para Convenios y Financieros.</t>
         </is>
       </c>
       <c r="G26" s="12" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
+          <t>Backlog del Chapter SD1. Convenios (sponsor Diana Riofrío y Patricia Romero); Financieros (sponsor Claro Gomez y Patricia Romero)</t>
         </is>
       </c>
       <c r="I26" s="7" t="n">
@@ -2344,12 +2344,12 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Renovación</t>
+          <t>Venta / Convenios y Financieros</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>(por confirmar)</t>
+          <t>Diana Riofrío, Patricia Romero (Convenios); Claro Gomez, Patricia Romero (Financieros)</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
@@ -2381,17 +2381,17 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Q-23</t>
+          <t>Q-25</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Venta</t>
+          <t>Vida Individual</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Sistema de incentivos orientados a la experiencia</t>
+          <t>Experiencia Postventa</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Orientar los incentivos de asesores hacia la experiencia</t>
+          <t>Mejorar la experiencia postventa de Vida Individual</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Diseño de un sistema de incentivos para asesores orientado a la experiencia (Back to Basics).</t>
+          <t>Rediseño de la experiencia postventa.</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
+          <t>Backlog del Chapter SD1 (sponsor Diana Riofrío)</t>
         </is>
       </c>
       <c r="I27" s="7" t="n">
@@ -2424,12 +2424,12 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Venta</t>
+          <t>Vida Individual / Posventa</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>(por confirmar)</t>
+          <t>Diana Riofrío</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
@@ -2461,17 +2461,17 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Q-24</t>
+          <t>Q-26</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Nuevo Modelo de Ventas</t>
+          <t>Ahorro Salud</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Convenios y Financieros — nuevo modelo de venta</t>
+          <t>Derivación eficiente MER</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2481,12 +2481,12 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Definir un nuevo modelo de venta para Convenios y Financieros</t>
+          <t>Hacer más eficiente la derivación (MER) en Ahorro Salud</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Nuevo modelo de venta para Convenios y Financieros.</t>
+          <t>Rediseño de la derivación eficiente MER.</t>
         </is>
       </c>
       <c r="G28" s="12" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Backlog del Chapter SD1. Convenios (sponsor Diana Riofrío y Patricia Romero); Financieros (sponsor Claro Gomez y Patricia Romero)</t>
+          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
         </is>
       </c>
       <c r="I28" s="7" t="n">
@@ -2504,12 +2504,12 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>Venta / Convenios y Financieros</t>
+          <t>Ahorro Salud</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>Diana Riofrío, Patricia Romero (Convenios); Claro Gomez, Patricia Romero (Financieros)</t>
+          <t>(por confirmar)</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
@@ -2538,173 +2538,13 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Q-25</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Vida Individual</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Experiencia Postventa</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Backlog (Chapter SD1)</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Mejorar la experiencia postventa de Vida Individual</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Rediseño de la experiencia postventa.</t>
-        </is>
-      </c>
-      <c r="G29" s="12" t="inlineStr">
-        <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Backlog del Chapter SD1 (sponsor Diana Riofrío)</t>
-        </is>
-      </c>
-      <c r="I29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>Vida Individual / Posventa</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="inlineStr">
-        <is>
-          <t>Diana Riofrío</t>
-        </is>
-      </c>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>(por confirmar)</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O29" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P29" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Q-26</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Ahorro Salud</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Derivación eficiente MER</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Backlog (Chapter SD1)</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Hacer más eficiente la derivación (MER) en Ahorro Salud</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Rediseño de la derivación eficiente MER.</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>Backlog</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>Backlog del Chapter SD1 (sin sprint asignado)</t>
-        </is>
-      </c>
-      <c r="I30" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>Ahorro Salud</t>
-        </is>
-      </c>
-      <c r="K30" s="5" t="inlineStr">
-        <is>
-          <t>(por confirmar)</t>
-        </is>
-      </c>
-      <c r="L30" s="5" t="inlineStr">
-        <is>
-          <t>(por confirmar)</t>
-        </is>
-      </c>
-      <c r="M30" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O30" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P30" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:P30"/>
+  <autoFilter ref="A4:P28"/>
   <mergeCells count="2">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I30">
+  <conditionalFormatting sqref="I5:I28">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
Beholder: 3 hitos (guía AMI diagramada, playbook B360, quick fix cobranzas)
- Q-1: agencia devolvió la 1ª guía resumida AMI diagramada (1/4) → 50%.
- Q-10: playbook de Bienestar 360 entregado (Stefanie).
- Q-4: quick fix de Stefanie — el correo de envío de datos de conciliación
  estaba errado y se corrigió → evita congelar dinero por falta de datos; 20%→35%.
Tablero + Excel + historial actualizados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WS4JWEE6ms3s7RzgD4pkSb
</commit_message>
<xml_diff>
--- a/reportes/Status_Proyectos_Behavioral_Design.xlsx
+++ b/reportes/Status_Proyectos_Behavioral_Design.xlsx
@@ -676,11 +676,11 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Diseño 1/4; roadmap reajustado −6 semanas; presentación del entregable 30/6; + flyers de venta (1×producto + comparativo)</t>
+          <t>Agencia devolvió la 1ª guía resumida AMI diagramada (1/4); roadmap reajustado −6 semanas; presentación del entregable 30/6; + flyers de venta (1×producto + comparativo)</t>
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
@@ -910,11 +910,11 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>12 entrevistas brokers/clientes B2B (entendimiento E2E del pago, pains de confirmación) → bajada/análisis → diseño de la nueva experiencia y pilotos → ejecutar piloto y definir experiencia final</t>
+          <t>12 entrevistas E2E + quick fix de Stefanie: el correo donde algunos proveedores enviaban los datos de conciliación estaba errado → corregido (evita congelar dinero por falta de datos); sigue diseño de la nueva experiencia y pilotos</t>
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
@@ -941,12 +941,12 @@
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>Track de diseño aprobado sin explorar la problemática</t>
+          <t>Track de diseño aprobado sin explorar la problemática (mitigándose: discovery + quick fix del correo de conciliación)</t>
         </is>
       </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Liberación de S/600k provisionados</t>
+          <t>Liberación de S/600k provisionados; el quick fix (correo de conciliación corregido) evita congelar dinero por falta de datos</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Implementado y en mantenimiento; cierre de playbook del programa + acompañamiento a la fase de mantenimiento</t>
+          <t>Implementado y en mantenimiento; playbook del programa entregado (Stefanie); acompañamiento a la fase de mantenimiento</t>
         </is>
       </c>
       <c r="I14" s="7" t="n">

</xml_diff>

<commit_message>
Cerrar códigos rojos: Q-6, Q-7 y Q-17 entregados, pasan a Done
Validador confirma 0 rojos activos (solo 1 amarillo: Q-28 sin
programar). Gantt y Excel regenerados desde el tablero.
</commit_message>
<xml_diff>
--- a/reportes/Status_Proyectos_Behavioral_Design.xlsx
+++ b/reportes/Status_Proyectos_Behavioral_Design.xlsx
@@ -941,14 +941,14 @@
           <t>Desk research + bench de estrategias de contacto en frío y caliente</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>En curso (4 días)</t>
+          <t>Entregado (4 días)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1013,14 +1013,14 @@
           <t>Validación con stakeholders</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Hoy (1 día)</t>
+          <t>Entregado (1 día)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1649,14 +1649,14 @@
           <t>Validación con stakeholders</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>En curso (3 días); pendiente check de Producto y equipo médico (nombre, coberturas, red, servicios)</t>
+          <t>Entregada (3 días); check de Producto y equipo médico completado (nombre, coberturas, red, servicios)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">

</xml_diff>